<commit_message>
fix: normalizar nomes de setor antes do matching (barras, espaços, case)
- Adicionada função _normalizar() que padroniza maiúsculas, remove barras
  no final, normaliza espaços ao redor de '/' e colapsa espaços duplos
- Agora 'BRONZE 1 / CORURIPE / FELIZ DESERTO/' bate com
  'Bronze 1 / CORURIPE / FELIZ DESERTO' mesmo com variações de formatação
- Removido alias VIPs (planilha agora usa o nome completo do setor)
- Atualizado metas.xlsx com nomes completos dos setores de 13707

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="crie uma planilha excel com ess" sheetId="1" r:id="rId5"/>
+    <sheet name="crie uma planilha excel com ess" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>SETOR</t>
   </si>
@@ -28,143 +33,143 @@
     <t>RPA</t>
   </si>
   <si>
-    <t>MULTIMARCA (%)</t>
-  </si>
-  <si>
-    <t>MULTIMARCA (Qtd)</t>
-  </si>
-  <si>
-    <t>CABELO (%)</t>
-  </si>
-  <si>
-    <t>CABELO (Qtd)</t>
-  </si>
-  <si>
-    <t>MAKE (%)</t>
-  </si>
-  <si>
-    <t>MAKE (Qtd)</t>
-  </si>
-  <si>
-    <t>BRONZE 1</t>
+    <t xml:space="preserve">MULTIMARCA (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIMARCA (Qtd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CABELO (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CABELO (Qtd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE (Qtd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRONZE 1 / CORURIPE / FELIZ DESERTO/</t>
   </si>
   <si>
     <t>NATALI</t>
   </si>
   <si>
-    <t>R$ 50.000,00</t>
-  </si>
-  <si>
-    <t>R$ 625,00</t>
-  </si>
-  <si>
-    <t>BRONZE 2</t>
+    <t xml:space="preserve">R$ 50.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 625,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRONZE 2 / PENEDO /</t>
   </si>
   <si>
     <t>EMANOELLE</t>
   </si>
   <si>
-    <t>R$ 55.000,00</t>
-  </si>
-  <si>
-    <t>R$ 611,11</t>
-  </si>
-  <si>
-    <t>BRONZE 3</t>
+    <t xml:space="preserve">R$ 55.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 611,11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRONZE 3 / PIAÇABUÇU / P.REAL / S.BRÁS / TEOTÔNIO /</t>
   </si>
   <si>
     <t>GISELLE</t>
   </si>
   <si>
-    <t>BRONZE 4</t>
+    <t xml:space="preserve">BRONZE 4 / SÃO SEBASTIÃO/ I. NOVA / OLHO'D /JUNQUEIRO/</t>
   </si>
   <si>
     <t>LUCIENE</t>
   </si>
   <si>
-    <t>R$ 687,50</t>
-  </si>
-  <si>
-    <t>PRATA 1</t>
+    <t xml:space="preserve">R$ 687,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRATA 1 / Penedo /</t>
   </si>
   <si>
     <t>LAÍS</t>
   </si>
   <si>
-    <t>R$ 125.000,00</t>
-  </si>
-  <si>
-    <t>R$ 1.190,48</t>
-  </si>
-  <si>
-    <t>PRATA 2</t>
+    <t xml:space="preserve">R$ 125.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 1.190,48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRATA 2 / Coruripe / Piaçabuçu / F. Deserto / São Sebastião /</t>
   </si>
   <si>
     <t>KAUANNE</t>
   </si>
   <si>
-    <t>R$ 160.000,00</t>
-  </si>
-  <si>
-    <t>R$ 1.333,33</t>
-  </si>
-  <si>
-    <t>PRATA 3</t>
+    <t xml:space="preserve">R$ 160.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 1.333,33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRATA 3 / I.Nova / Junqueiro / Olho D' Agua / Porto Real / São Brás / Teotônio</t>
   </si>
   <si>
     <t>SABRINA</t>
   </si>
   <si>
-    <t>R$ 140.000,00</t>
-  </si>
-  <si>
-    <t>R$ 1.217,39</t>
-  </si>
-  <si>
-    <t>OURO</t>
+    <t xml:space="preserve">R$ 140.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 1.217,39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OURO / Penedo /</t>
   </si>
   <si>
     <t>LETÍCIA</t>
   </si>
   <si>
-    <t>R$ 360.000,00</t>
-  </si>
-  <si>
-    <t>R$ 2.400,00</t>
-  </si>
-  <si>
-    <t>PLATINA</t>
+    <t xml:space="preserve">R$ 360.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 2.400,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLATINA / Penedo /</t>
   </si>
   <si>
     <t>NATHÁLIA</t>
   </si>
   <si>
-    <t>R$ 320.000,00</t>
-  </si>
-  <si>
-    <t>R$ 3.800,00</t>
-  </si>
-  <si>
-    <t>VIPs</t>
+    <t xml:space="preserve">R$ 320.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 3.800,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPERVISORA DE RELACIONAMENTO PENEDO</t>
   </si>
   <si>
     <t>GÉSSICA</t>
   </si>
   <si>
-    <t>R$ 700.000,00</t>
-  </si>
-  <si>
-    <t>R$ 24.000,00</t>
+    <t xml:space="preserve">R$ 700.000,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R$ 24.000,00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
+      <sz val="10.000000"/>
+      <color indexed="64"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -179,43 +184,330 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -272,7 +564,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -298,7 +590,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -375,7 +667,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -405,15 +697,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="53.421875"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -461,28 +758,28 @@
         <v>13</v>
       </c>
       <c r="D2" s="1">
-        <v>80.0</v>
+        <v>80</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F2" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G2" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="H2" s="2">
-        <v>0.36</v>
+        <v>0.35999999999999999</v>
       </c>
       <c r="I2" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="J2" s="2">
-        <v>0.35</v>
+        <v>0.34999999999999998</v>
       </c>
       <c r="K2" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -496,28 +793,28 @@
         <v>17</v>
       </c>
       <c r="D3" s="1">
-        <v>90.0</v>
+        <v>90</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F3" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G3" s="1">
-        <v>73.0</v>
+        <v>73</v>
       </c>
       <c r="H3" s="2">
-        <v>0.36</v>
+        <v>0.35999999999999999</v>
       </c>
       <c r="I3" s="1">
-        <v>36.0</v>
+        <v>36</v>
       </c>
       <c r="J3" s="2">
-        <v>0.35</v>
+        <v>0.34999999999999998</v>
       </c>
       <c r="K3" s="1">
-        <v>35.0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -531,28 +828,28 @@
         <v>13</v>
       </c>
       <c r="D4" s="1">
-        <v>80.0</v>
+        <v>80</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G4" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2">
-        <v>0.36</v>
+        <v>0.35999999999999999</v>
       </c>
       <c r="I4" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="J4" s="2">
-        <v>0.35</v>
+        <v>0.34999999999999998</v>
       </c>
       <c r="K4" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -566,28 +863,28 @@
         <v>17</v>
       </c>
       <c r="D5" s="1">
-        <v>80.0</v>
+        <v>80</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F5" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G5" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2">
-        <v>0.36</v>
+        <v>0.35999999999999999</v>
       </c>
       <c r="I5" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="J5" s="2">
-        <v>0.35</v>
+        <v>0.34999999999999998</v>
       </c>
       <c r="K5" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -601,28 +898,28 @@
         <v>26</v>
       </c>
       <c r="D6" s="1">
-        <v>105.0</v>
+        <v>105</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G6" s="1">
-        <v>84.0</v>
+        <v>84</v>
       </c>
       <c r="H6" s="2">
         <v>0.37</v>
       </c>
       <c r="I6" s="1">
-        <v>43.0</v>
+        <v>43</v>
       </c>
       <c r="J6" s="2">
         <v>0.37</v>
       </c>
       <c r="K6" s="1">
-        <v>43.0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -636,28 +933,28 @@
         <v>30</v>
       </c>
       <c r="D7" s="1">
-        <v>120.0</v>
+        <v>120</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F7" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G7" s="1">
-        <v>95.0</v>
+        <v>95</v>
       </c>
       <c r="H7" s="2">
         <v>0.37</v>
       </c>
       <c r="I7" s="1">
-        <v>48.0</v>
+        <v>48</v>
       </c>
       <c r="J7" s="2">
         <v>0.37</v>
       </c>
       <c r="K7" s="1">
-        <v>48.0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -671,28 +968,28 @@
         <v>34</v>
       </c>
       <c r="D8" s="1">
-        <v>115.0</v>
+        <v>115</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>35</v>
       </c>
       <c r="F8" s="2">
-        <v>0.73</v>
+        <v>0.72999999999999998</v>
       </c>
       <c r="G8" s="1">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="H8" s="2">
         <v>0.37</v>
       </c>
       <c r="I8" s="1">
-        <v>46.0</v>
+        <v>46</v>
       </c>
       <c r="J8" s="2">
         <v>0.37</v>
       </c>
       <c r="K8" s="1">
-        <v>46.0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
@@ -706,7 +1003,7 @@
         <v>38</v>
       </c>
       <c r="D9" s="1">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>39</v>
@@ -715,19 +1012,19 @@
         <v>0.75</v>
       </c>
       <c r="G9" s="1">
-        <v>120.0</v>
+        <v>120</v>
       </c>
       <c r="H9" s="2">
-        <v>0.39</v>
+        <v>0.39000000000000001</v>
       </c>
       <c r="I9" s="1">
-        <v>62.0</v>
+        <v>62</v>
       </c>
       <c r="J9" s="2">
-        <v>0.42</v>
+        <v>0.41999999999999998</v>
       </c>
       <c r="K9" s="1">
-        <v>67.0</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10">
@@ -741,28 +1038,28 @@
         <v>42</v>
       </c>
       <c r="D10" s="1">
-        <v>72.0</v>
+        <v>72</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>43</v>
       </c>
       <c r="F10" s="2">
-        <v>0.8</v>
+        <v>0.80000000000000004</v>
       </c>
       <c r="G10" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2">
-        <v>0.45</v>
+        <v>0.45000000000000001</v>
       </c>
       <c r="I10" s="1">
-        <v>37.0</v>
+        <v>37</v>
       </c>
       <c r="J10" s="2">
         <v>0.5</v>
       </c>
       <c r="K10" s="1">
-        <v>41.0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11">
@@ -776,31 +1073,34 @@
         <v>46</v>
       </c>
       <c r="D11" s="1">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>47</v>
       </c>
       <c r="F11" s="2">
-        <v>0.8</v>
+        <v>0.80000000000000004</v>
       </c>
       <c r="G11" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="H11" s="2">
-        <v>0.65</v>
+        <v>0.65000000000000002</v>
       </c>
       <c r="I11" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="J11" s="2">
-        <v>0.6</v>
+        <v>0.59999999999999998</v>
       </c>
       <c r="K11" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: corrigir nomes dos setores 13706 para bater com a planilha real
- OURO / Palmeira / -> OURO Palmeira
- PRATA 2 com cidades abreviadas conforme planilha real
- Adiciona VIPS / PLATINA /Palmeira com mesmas metas da Supervisora de Relacionamento Palmeira

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -330,7 +330,7 @@
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="53.421875" customWidth="1" min="1" max="1"/>
@@ -826,7 +826,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OURO / Palmeira /</t>
+          <t>OURO Palmeira</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PRATA 2 / Major / Estrela de Alagoas / Minador do Negrao / Cacimbinhas / Quebrangulo / Igaci /</t>
+          <t>PRATA 2 / Major / Cacimbinhas / Estrela / Quebrangulo / Minador /Igaci/</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1035,6 +1035,49 @@
         <v>0.6</v>
       </c>
       <c r="K16" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>VIPS / PLATINA /Palmeira</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>JORDELLE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R$ 420.000,00</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>60</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>R$ 7.000,00</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G17" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I17" t="n">
+        <v>24</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K17" t="n">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: atualizar metas das supervisoras 13706 e 13707
Atualiza Receita, Clientes Ativos e RPA para todas as supervisoras
das gerências 13706 (DANIELLE, BRUNA, EDNA, LUAN, JORDELLE) e 13707
(LETÍCIA, NATHÁLIA, LAÍS, KAUANNE, SABRINA, NATALI, KARINE, GISELLE,
LUCIENE, GÉSSICA). Remove linha duplicada 'SUPERVISORA DE
RELACIONAMENTO PALMEIRA' (JORDELLE) — meta consolidada em
'VIPS / PLATINA /Palmeira'. Colunas Multi/Cabelo/Make preservadas.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -330,7 +330,7 @@
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="53.421875" customWidth="1" min="1" max="1"/>
@@ -406,15 +406,15 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 25.000,00</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>R$ 700,00</t>
+          <t>R$ 384,00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -449,15 +449,15 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 30.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 700,00</t>
+          <t>R$ 375,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,15 +492,15 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 30.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 700,00</t>
+          <t>R$ 428,57</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -535,15 +535,15 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 65.000,00</t>
+          <t>R$ 30.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 700,00</t>
+          <t>R$ 441,18</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,15 +578,15 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 160.000,00</t>
+          <t>R$ 110.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,15 +621,15 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>R$ 160.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.300,00</t>
+          <t>R$ 1.454,55</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,15 +664,15 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 180.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.250,00</t>
+          <t>R$ 1.363,64</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 450.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.500,00</t>
+          <t>R$ 1.764,71</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 380.000,00</t>
+          <t>R$ 260.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 4.000,00</t>
+          <t>R$ 3.376,62</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.286.000,00</t>
+          <t>R$ 700.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>R$ 35.000,00</t>
+          <t>R$ 25.000,00</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -836,7 +836,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 320.000,00</t>
+          <t>R$ 230.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -844,7 +844,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>R$ 2.500,00</t>
+          <t>R$ 1.916,00</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -879,15 +879,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 70.000,00</t>
+          <t>R$ 30.000,00</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 700,00</t>
+          <t>R$ 344,83</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -922,15 +922,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 190.000,00</t>
+          <t>R$ 100.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>R$ 1.350,00</t>
+          <t>R$ 1.111,11</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -965,15 +965,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 170.000,00</t>
+          <t>R$ 110.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 1.250,00</t>
+          <t>R$ 1.222,22</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -998,7 +998,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SUPERVISORA DE RELACIONAMENTO PALMEIRA</t>
+          <t>VIPS / PLATINA /Palmeira</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 420.000,00</t>
+          <t>R$ 290.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 7.000,00</t>
+          <t>R$ 4.833,33</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1035,49 +1035,6 @@
         <v>0.6</v>
       </c>
       <c r="K16" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>VIPS / PLATINA /Palmeira</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>JORDELLE</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>R$ 420.000,00</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>60</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>R$ 7.000,00</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G17" t="n">
-        <v>30</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="I17" t="n">
-        <v>24</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K17" t="n">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: atualizar metas do novo ciclo (Receita, RPA e Clientes Ativos)
Atualiza as metas dos 15 setores das 2 gerencias (Penedo/Matriz e Palmeira/Filial) para o novo ciclo. Apenas RECEITA, ATIVO e RPA foram alterados; metas de IAF (multimarca/cabelo/make) e supervisoras mantidas.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -406,15 +406,15 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>R$ 25.000,00</t>
+          <t>R$ 35.000,00</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>R$ 384,00</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -449,15 +449,15 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 35.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 375,00</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,15 +492,15 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 35.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 428,57</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -535,15 +535,15 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 35.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 441,18</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,15 +578,15 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 110.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,15 +621,15 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 160.000,00</t>
+          <t>R$ 170.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.454,55</t>
+          <t>R$ 1.250,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,15 +664,15 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>R$ 160.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.363,64</t>
+          <t>R$ 1.250,00</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>R$ 350.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.764,71</t>
+          <t>R$ 2.000,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,15 +750,15 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 260.000,00</t>
+          <t>R$ 270.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 3.376,62</t>
+          <t>R$ 3.300,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -836,15 +836,15 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 230.000,00</t>
+          <t>R$ 210.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>R$ 1.916,00</t>
+          <t>R$ 1.600,00</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -879,15 +879,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 40.000,00</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 344,83</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -922,15 +922,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 100.000,00</t>
+          <t>R$ 135.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>R$ 1.111,11</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -965,15 +965,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 110.000,00</t>
+          <t>R$ 125.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 1.222,22</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 290.000,00</t>
+          <t>R$ 305.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 4.833,33</t>
+          <t>R$ 5.000,00</t>
         </is>
       </c>
       <c r="F16" t="n">

</xml_diff>

<commit_message>
chore: atualiza metas do Ciclo 9 (Receita, Ativos e RPA por setor)
Aplica as novas metas das gerencias 13706 e 13707 a partir da planilha
META CICLO 9 CADU.xlsx nos 15 setores. Multimarca/Cabelo/Make mantidos.
Linha VIPS PENEDO aplicada ao setor SUPERVISORA DE RELACIONAMENTO PENEDO
(nome preservado); setor novo "13706 -FVC" nao adicionado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -406,7 +406,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>R$ 35.000,00</t>
+          <t>R$ 21.000,00</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
@@ -414,7 +414,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>R$ 550,00</t>
+          <t>R$ 400,00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -449,7 +449,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 35.000,00</t>
+          <t>R$ 21.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
@@ -457,7 +457,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 550,00</t>
+          <t>R$ 400,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 35.000,00</t>
+          <t>R$ 28.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
@@ -500,7 +500,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 550,00</t>
+          <t>R$ 400,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 35.000,00</t>
+          <t>R$ 28.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 550,00</t>
+          <t>R$ 400,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,15 +578,15 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>R$ 110.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.000,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,15 +621,15 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 170.000,00</t>
+          <t>R$ 130.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.250,00</t>
+          <t>R$ 1.000,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,15 +664,15 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 160.000,00</t>
+          <t>R$ 120.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.250,00</t>
+          <t>R$ 1.000,00</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,15 +707,15 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 350.000,00</t>
+          <t>R$ 330.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.000,00</t>
+          <t>R$ 1.900,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 270.000,00</t>
+          <t>R$ 240.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 3.300,00</t>
+          <t>R$ 2.500,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 700.000,00</t>
+          <t>R$ 807.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -836,15 +836,15 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 210.000,00</t>
+          <t>R$ 190.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>R$ 1.600,00</t>
+          <t>R$ 2.000,00</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -879,15 +879,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 40.000,00</t>
+          <t>R$ 30.000,00</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 550,00</t>
+          <t>R$ 450,00</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -922,15 +922,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 135.000,00</t>
+          <t>R$ 120.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.150,00</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -965,15 +965,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 125.000,00</t>
+          <t>R$ 115.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.150,00</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 305.000,00</t>
+          <t>R$ 315.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 5.000,00</t>
+          <t>R$ 4.900,00</t>
         </is>
       </c>
       <c r="F16" t="n">

</xml_diff>

<commit_message>
feat(metas): atualiza metas do ciclo 10 e troca supervisoras de Penedo
- metas.xlsx: aplica receita/ativos/RPA do ciclo 10 nos 15 setores
  (colunas MULTIMARCA/CABELO/MAKE preservadas)
- Platina/Penedo: NATHALIA -> ANALUIZA
- Bronze 4/Penedo: LUCIENE -> RODRIGO
- config.py: mapeia Slack IDs de ANALUIZA e RODRIGO no mapa embutido

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -406,11 +406,11 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>R$ 21.000,00</t>
+          <t>R$ 37.000,00</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
@@ -449,15 +449,15 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 21.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 400,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 28.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
@@ -500,7 +500,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 400,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -530,12 +530,12 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>LUCIENE</t>
+          <t>RODRIGO</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 28.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 400,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,15 +578,15 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 110.000,00</t>
+          <t>R$ 145.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.000,00</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,15 +621,15 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 130.000,00</t>
+          <t>R$ 188.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.000,00</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,15 +664,15 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 120.000,00</t>
+          <t>R$ 175.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.000,00</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,15 +707,15 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 330.000,00</t>
+          <t>R$ 437.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.900,00</t>
+          <t>R$ 2.500,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -745,12 +745,12 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>NATHÁLIA</t>
+          <t>ANALUIZA</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 240.000,00</t>
+          <t>R$ 380.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.500,00</t>
+          <t>R$ 3.800,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 807.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>R$ 25.000,00</t>
+          <t>R$ 26.000,00</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -836,7 +836,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 190.000,00</t>
+          <t>R$ 200.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -879,7 +879,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 50.000,00</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -922,11 +922,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 120.000,00</t>
+          <t>R$ 130.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -965,11 +965,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 115.000,00</t>
+          <t>R$ 130.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 315.000,00</t>
+          <t>R$ 400.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">

</xml_diff>

<commit_message>
chore: atualiza metas do Ciclo 11 (Receita, Ativos e RPA por setor)
Aplica as metas do Ciclo 11 nos 15 setores a partir de
"Metas Ciclo 11 Cadu.xlsx". Apenas RECEITA, ATIVO e RPA mudam;
as colunas de multimarca, cabelo e make ficam inalteradas.

Ativos alterados: Bronze 2 / Penedo (75 -> 85) e
Prata 2 / Penedo (120 -> 125). RPA = receita / ativos.

Backup do estado anterior em metas.xlsx.bak_pre_ciclo11.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -406,7 +406,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>R$ 37.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
@@ -414,7 +414,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>R$ 400,00</t>
+          <t>R$ 600,00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -449,15 +449,15 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 45.000,00</t>
+          <t>R$ 70.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 500,00</t>
+          <t>R$ 823,53</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 45.000,00</t>
+          <t>R$ 60.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
@@ -500,7 +500,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 500,00</t>
+          <t>R$ 800,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 45.000,00</t>
+          <t>R$ 55.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 500,00</t>
+          <t>R$ 733,33</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,7 +578,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 145.000,00</t>
+          <t>R$ 133.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.156,52</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,15 +621,15 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 188.000,00</t>
+          <t>R$ 160.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.280,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 175.000,00</t>
+          <t>R$ 145.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.260,87</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 437.000,00</t>
+          <t>R$ 390.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.500,00</t>
+          <t>R$ 2.392,64</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 380.000,00</t>
+          <t>R$ 310.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 3.800,00</t>
+          <t>R$ 3.875,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 800.000,00</t>
+          <t>R$ 680.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>R$ 26.000,00</t>
+          <t>R$ 24.285,71</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -836,7 +836,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>R$ 180.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -879,7 +879,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 50.000,00</t>
+          <t>R$ 80.000,00</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -887,7 +887,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 450,00</t>
+          <t>R$ 800,00</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 130.000,00</t>
+          <t>R$ 115.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>R$ 1.150,00</t>
+          <t>R$ 1.210,53</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -965,7 +965,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 130.000,00</t>
+          <t>R$ 106.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 1.150,00</t>
+          <t>R$ 1.115,79</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 400.000,00</t>
+          <t>R$ 350.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 4.900,00</t>
+          <t>R$ 5.833,33</t>
         </is>
       </c>
       <c r="F16" t="n">

</xml_diff>

<commit_message>
chore: atualiza metas do Ciclo 12 e troca supervisoras de Bronze 1/4
Aplica as metas do Ciclo 12 nos 15 setores a partir de
"metas ciclo 12 CADU.xlsx". Apenas RECEITA, ATIVO e RPA mudam;
as colunas de multimarca, cabelo e make ficam inalteradas.

O R$/ATIVO da planilha nao e receita / ativos como nos ciclos
anteriores: vem como meta arredondada propria (ex.: VIPs Penedo
700.000/28 = 25.000, mas a planilha pede 23.000). Usado o valor
da planilha.

Receita total 2.879.000 -> 2.864.000; ativos 1.376 -> 1.457.

Troca de supervisoras enquanto a Natali esta de ferias:
Bronze 1 / Coruripe passa de NATALI para RODRIGO, e Bronze 4 /
Sao Sebastiao passa de RODRIGO para LUCIENE. As metas seguem o
setor, nao a pessoa. Ambos ja estao no SLACK_USER_MAP do Render,
entao o card do Slack vai para o destinatario certo; NATALI
segue mapeada para quando voltar.

Backups do estado anterior em metas.xlsx.bak_pre_ciclo12 e
metas.xlsx.bak_pre_troca_sup.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -401,7 +401,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>NATALI</t>
+          <t>RODRIGO</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -410,11 +410,11 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>R$ 600,00</t>
+          <t>R$ 400,00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -449,15 +449,15 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 70.000,00</t>
+          <t>R$ 50.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 823,53</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,15 +492,15 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 50.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 800,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -530,20 +530,20 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>RODRIGO</t>
+          <t>LUCIENE</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 55.000,00</t>
+          <t>R$ 50.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 733,33</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,7 +578,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 133.000,00</t>
+          <t>R$ 130.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.156,52</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,15 +621,15 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 160.000,00</t>
+          <t>R$ 170.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.280,00</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -668,11 +668,11 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.260,87</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -711,11 +711,11 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.392,64</t>
+          <t>R$ 2.100,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,15 +750,15 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 310.000,00</t>
+          <t>R$ 305.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 3.875,00</t>
+          <t>R$ 3.500,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 680.000,00</t>
+          <t>R$ 700.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>R$ 24.285,71</t>
+          <t>R$ 23.000,00</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -840,11 +840,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>R$ 2.000,00</t>
+          <t>R$ 1.800,00</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -883,11 +883,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 800,00</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -926,11 +926,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>R$ 1.210,53</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -965,7 +965,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 106.000,00</t>
+          <t>R$ 104.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 1.115,79</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1012,11 +1012,11 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 5.833,33</t>
+          <t>R$ 4.500,00</t>
         </is>
       </c>
       <c r="F16" t="n">

</xml_diff>

<commit_message>
feat(metas): metas do Ciclo 13 nos 15 setores
Receita, meta de ativos e R$/ativo vindos da planilha do ciclo.
RPA copiado da coluna R$/ATIVO, nao recalculado como receita / ativos.
Multimarca, cabelo e make ficam inalterados.

A meta de ativos veio igual a do Ciclo 12 em todos os setores.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GnC7VoWKTB23HJRQQm7Xgp
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -449,7 +449,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 50.000,00</t>
+          <t>R$ 70.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
@@ -457,7 +457,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 500,00</t>
+          <t>R$ 600,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 50.000,00</t>
+          <t>R$ 60.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
@@ -500,7 +500,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 500,00</t>
+          <t>R$ 600,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 50.000,00</t>
+          <t>R$ 60.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 500,00</t>
+          <t>R$ 600,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,7 +578,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 130.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,7 +621,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 170.000,00</t>
+          <t>R$ 200.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
@@ -629,7 +629,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.300,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 145.000,00</t>
+          <t>R$ 160.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.200,00</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 390.000,00</t>
+          <t>R$ 420.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.100,00</t>
+          <t>R$ 2.200,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 305.000,00</t>
+          <t>R$ 350.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 3.500,00</t>
+          <t>R$ 3.900,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 700.000,00</t>
+          <t>R$ 750.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>R$ 23.000,00</t>
+          <t>R$ 25.000,00</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -836,7 +836,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 180.000,00</t>
+          <t>R$ 215.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -844,7 +844,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>R$ 1.800,00</t>
+          <t>R$ 1.900,00</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -887,7 +887,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 550,00</t>
+          <t>R$ 650,00</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 115.000,00</t>
+          <t>R$ 125.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.150,00</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -965,7 +965,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 104.000,00</t>
+          <t>R$ 120.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 1.100,00</t>
+          <t>R$ 1.150,00</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 350.000,00</t>
+          <t>R$ 400.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 4.500,00</t>
+          <t>R$ 4.800,00</t>
         </is>
       </c>
       <c r="F16" t="n">

</xml_diff>